<commit_message>
Updated dashboard overlay spreadsheet
</commit_message>
<xml_diff>
--- a/EEE2000-metadata_mapping.xlsx
+++ b/EEE2000-metadata_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rhys.r.evans/Documents/CEDA/CCI/cci_data_bridge_inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stfc365-my.sharepoint.com/personal/alison_waterfall_stfc_ac_uk/Documents/Documents/GitHub/cci_data_bridge_inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AAB98B8-BC09-4544-B40F-5DB8A5DD5A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{0AAB98B8-BC09-4544-B40F-5DB8A5DD5A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C817DEB-570A-4AB7-A3FA-074D47EFF721}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="2220" windowWidth="32520" windowHeight="17580" activeTab="1" xr2:uid="{B9DA58AC-C110-4CBA-A19B-6F37B44EEA38}"/>
+    <workbookView xWindow="42060" yWindow="4590" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{B9DA58AC-C110-4CBA-A19B-6F37B44EEA38}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapping" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1834" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2424" uniqueCount="591">
   <si>
     <t>Dataset 1</t>
   </si>
@@ -1874,6 +1874,282 @@
   </si>
   <si>
     <t>https://catalogue.ceda.ac.uk/uuid/6429d1aafe1e43b9b414e4a5a7f8b903</t>
+  </si>
+  <si>
+    <t>Light Gradient Boosting</t>
+  </si>
+  <si>
+    <t>Bias correction</t>
+  </si>
+  <si>
+    <t>Retrieval of dust</t>
+  </si>
+  <si>
+    <t>Classification of irrigation</t>
+  </si>
+  <si>
+    <t>Cloud mask</t>
+  </si>
+  <si>
+    <t>Determine cloud parameters</t>
+  </si>
+  <si>
+    <t>Convolutional Neural Network</t>
+  </si>
+  <si>
+    <t>Deep Learning – convolutional neural networks</t>
+  </si>
+  <si>
+    <t>Combining SAR and optical</t>
+  </si>
+  <si>
+    <t>Uncertainty classification probabilities</t>
+  </si>
+  <si>
+    <t>GHGs</t>
+  </si>
+  <si>
+    <t>Cloud coverage pre-filtering</t>
+  </si>
+  <si>
+    <t>Quality-filtering and predicting bias</t>
+  </si>
+  <si>
+    <t>Extreme Gradient Boosting</t>
+  </si>
+  <si>
+    <t>Quality-filtering</t>
+  </si>
+  <si>
+    <t>HRLC</t>
+  </si>
+  <si>
+    <t>K-means clustering</t>
+  </si>
+  <si>
+    <t>Binary water extraction from SAR</t>
+  </si>
+  <si>
+    <t>Weak Supervision</t>
+  </si>
+  <si>
+    <t>Pretraining classification with thematic maps</t>
+  </si>
+  <si>
+    <t>Siamese Multi-Layer Perceptron</t>
+  </si>
+  <si>
+    <t>Deep Learning – feed-forward neural networks</t>
+  </si>
+  <si>
+    <t>Decision fusion between optical and SAR</t>
+  </si>
+  <si>
+    <t>Vision Transformer</t>
+  </si>
+  <si>
+    <t>Deep Learning – transformers</t>
+  </si>
+  <si>
+    <t>Classification of land cover from optical</t>
+  </si>
+  <si>
+    <t>Encoder-Decoder Transformer</t>
+  </si>
+  <si>
+    <t>Classification of land cover from SAR</t>
+  </si>
+  <si>
+    <t>Ice Sheets (Antarctica)</t>
+  </si>
+  <si>
+    <t>Holistically-Nested Edge Detection</t>
+  </si>
+  <si>
+    <t>Delineate grounding lines of ice shelves</t>
+  </si>
+  <si>
+    <t>U-Net Convolutional Neural Network</t>
+  </si>
+  <si>
+    <t>Delineate ice shelf coastlines</t>
+  </si>
+  <si>
+    <t>Combining SAR and altimetry data</t>
+  </si>
+  <si>
+    <t>Ice Sheets (Greenland)</t>
+  </si>
+  <si>
+    <t>Classification of supraglacial lakes</t>
+  </si>
+  <si>
+    <t>Combining SAR and optical data</t>
+  </si>
+  <si>
+    <t>Back Propagation Neural Network</t>
+  </si>
+  <si>
+    <t>Gap-filling</t>
+  </si>
+  <si>
+    <t>Producing gap-filled LSWT/ LIC dataset</t>
+  </si>
+  <si>
+    <t>Multi-layer Perceptron Neural Network</t>
+  </si>
+  <si>
+    <t>Define water level relation with altimetry</t>
+  </si>
+  <si>
+    <t>First-order water detection</t>
+  </si>
+  <si>
+    <t>Resolution enhancement</t>
+  </si>
+  <si>
+    <t>Transfer to various spatial resolution data</t>
+  </si>
+  <si>
+    <t>Quantify classification uncertainty per pixel</t>
+  </si>
+  <si>
+    <t>Gradient Boosting</t>
+  </si>
+  <si>
+    <t>Reduce hyperspectral dimensionality</t>
+  </si>
+  <si>
+    <t>Encoder Transformer</t>
+  </si>
+  <si>
+    <t>Change detection benchmarking</t>
+  </si>
+  <si>
+    <t>Classify reflectance into land cover types</t>
+  </si>
+  <si>
+    <t>LST</t>
+  </si>
+  <si>
+    <t>Retrieve LST from brightness temperature</t>
+  </si>
+  <si>
+    <t>Generate fractional vegetation cover</t>
+  </si>
+  <si>
+    <t>Estimate retrieval uncertainty</t>
+  </si>
+  <si>
+    <t>Cluster retrieval errors for calibration</t>
+  </si>
+  <si>
+    <t>Downscaling microwave for merged product</t>
+  </si>
+  <si>
+    <t>Feed-forward Neural Network</t>
+  </si>
+  <si>
+    <t>Retrieve water Inherent Optical Properties</t>
+  </si>
+  <si>
+    <t>Atmospheric correction</t>
+  </si>
+  <si>
+    <t>Predict ozone profiles</t>
+  </si>
+  <si>
+    <t>Grouping of conditions for separate models</t>
+  </si>
+  <si>
+    <t>Permafrost</t>
+  </si>
+  <si>
+    <t>Generate land cover unit parameters</t>
+  </si>
+  <si>
+    <t>Processing super-resolution land cover units</t>
+  </si>
+  <si>
+    <t>Use case on drivers</t>
+  </si>
+  <si>
+    <t>Use case on drivers and impacts</t>
+  </si>
+  <si>
+    <t>Use case on impacts</t>
+  </si>
+  <si>
+    <t>Phyto</t>
+  </si>
+  <si>
+    <t>Derive phytoplankton pigments</t>
+  </si>
+  <si>
+    <t>Precursors</t>
+  </si>
+  <si>
+    <t>Convert radiance into column abundance</t>
+  </si>
+  <si>
+    <t>SAGE</t>
+  </si>
+  <si>
+    <t>Diffusion Models</t>
+  </si>
+  <si>
+    <t>Deep Learning – generative models</t>
+  </si>
+  <si>
+    <t>Enhance resolution of old microwave data</t>
+  </si>
+  <si>
+    <t>Extract waveform clusters for training</t>
+  </si>
+  <si>
+    <t>Cross-channel ice signature identification</t>
+  </si>
+  <si>
+    <t>Set waveform cutoff for radar retrieval</t>
+  </si>
+  <si>
+    <t>Graph Neural Network</t>
+  </si>
+  <si>
+    <t>Deep Learning – graph neural networks</t>
+  </si>
+  <si>
+    <t>Processing old microwave records to extend</t>
+  </si>
+  <si>
+    <t>Sea State</t>
+  </si>
+  <si>
+    <t>Support Vector Machine</t>
+  </si>
+  <si>
+    <t>Estimate significant wave height</t>
+  </si>
+  <si>
+    <t>Sea Surface Salinity</t>
+  </si>
+  <si>
+    <t>Remove radio-frequency interference</t>
+  </si>
+  <si>
+    <t>Remove geophysical effects</t>
+  </si>
+  <si>
+    <t>Attribution of SST variability modelling</t>
+  </si>
+  <si>
+    <t>Long Short Term Memory</t>
+  </si>
+  <si>
+    <t>Deep Learning – recurrent neural networks</t>
+  </si>
+  <si>
+    <t>Predicting future SST modelling</t>
   </si>
 </sst>
 </file>
@@ -1945,18 +2221,15 @@
       <color rgb="FF212529"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF467886"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF212529"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2105,7 +2378,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2159,27 +2432,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2194,31 +2446,77 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2536,36 +2834,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CC0B67C-1229-4907-A814-DF79422D0B81}">
   <dimension ref="A1:M170"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5" customWidth="1"/>
-    <col min="3" max="3" width="30.1640625" customWidth="1"/>
-    <col min="4" max="4" width="38.5" customWidth="1"/>
-    <col min="5" max="5" width="23.5" customWidth="1"/>
-    <col min="6" max="6" width="23.5" style="6" customWidth="1"/>
-    <col min="7" max="7" width="30.5" style="9" customWidth="1"/>
-    <col min="8" max="8" width="30.5" style="12" customWidth="1"/>
-    <col min="9" max="9" width="42.83203125" style="4" customWidth="1"/>
-    <col min="10" max="10" width="19.5" style="4" customWidth="1"/>
-    <col min="11" max="11" width="19.5" customWidth="1"/>
-    <col min="12" max="12" width="23.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="47.1640625" style="8" customWidth="1"/>
+    <col min="1" max="1" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="4" max="4" width="38.42578125" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" style="9" customWidth="1"/>
+    <col min="8" max="8" width="30.42578125" style="12" customWidth="1"/>
+    <col min="9" max="9" width="42.85546875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="19.42578125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" customWidth="1"/>
+    <col min="12" max="12" width="23.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="47.140625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="44" t="s">
         <v>2</v>
       </c>
       <c r="I1" s="14" t="s">
@@ -2575,7 +2873,7 @@
       <c r="K1" s="3"/>
       <c r="M1" s="17"/>
     </row>
-    <row r="2" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2594,8 +2892,8 @@
       <c r="F2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="31"/>
-      <c r="H2" s="33"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="45"/>
       <c r="I2" s="15" t="s">
         <v>10</v>
       </c>
@@ -2612,7 +2910,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -2653,7 +2951,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -2694,11 +2992,11 @@
         <v>229</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
     </row>
-    <row r="6" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -2739,7 +3037,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -2780,7 +3078,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -2821,11 +3119,11 @@
         <v>201</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B9" s="19"/>
       <c r="C9" s="19"/>
     </row>
-    <row r="10" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -2866,7 +3164,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -2907,7 +3205,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -2948,7 +3246,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -2989,7 +3287,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>42</v>
       </c>
@@ -3030,7 +3328,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -3071,7 +3369,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -3112,7 +3410,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -3153,7 +3451,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -3194,7 +3492,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -3235,7 +3533,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -3276,7 +3574,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -3317,7 +3615,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -3358,7 +3656,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -3399,7 +3697,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -3440,7 +3738,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>42</v>
       </c>
@@ -3481,7 +3779,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>42</v>
       </c>
@@ -3522,7 +3820,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>42</v>
       </c>
@@ -3563,7 +3861,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -3604,7 +3902,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -3645,7 +3943,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -3686,7 +3984,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -3727,7 +4025,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -3768,11 +4066,11 @@
         <v>233</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B33" s="19"/>
       <c r="C33" s="19"/>
     </row>
-    <row r="34" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -3813,7 +4111,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -3854,11 +4152,11 @@
         <v>220</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B36" s="19"/>
       <c r="C36" s="19"/>
     </row>
-    <row r="37" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -3899,7 +4197,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>74</v>
       </c>
@@ -3940,7 +4238,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -3981,7 +4279,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -4022,7 +4320,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>74</v>
       </c>
@@ -4063,7 +4361,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>74</v>
       </c>
@@ -4104,7 +4402,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>74</v>
       </c>
@@ -4145,7 +4443,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>85</v>
       </c>
@@ -4186,7 +4484,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>85</v>
       </c>
@@ -4227,7 +4525,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>85</v>
       </c>
@@ -4268,7 +4566,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>85</v>
       </c>
@@ -4309,7 +4607,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>85</v>
       </c>
@@ -4350,7 +4648,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>85</v>
       </c>
@@ -4391,7 +4689,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>85</v>
       </c>
@@ -4432,7 +4730,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
       <c r="B51" s="19">
         <v>43501</v>
@@ -4471,7 +4769,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>85</v>
       </c>
@@ -4512,7 +4810,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>85</v>
       </c>
@@ -4553,7 +4851,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>85</v>
       </c>
@@ -4594,7 +4892,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>85</v>
       </c>
@@ -4635,12 +4933,12 @@
         <v>236</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="10"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
     </row>
-    <row r="57" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>100</v>
       </c>
@@ -4681,7 +4979,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>100</v>
       </c>
@@ -4722,7 +5020,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>100</v>
       </c>
@@ -4763,7 +5061,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>100</v>
       </c>
@@ -4804,7 +5102,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>100</v>
       </c>
@@ -4845,7 +5143,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>100</v>
       </c>
@@ -4886,7 +5184,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>100</v>
       </c>
@@ -4927,7 +5225,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>100</v>
       </c>
@@ -4968,7 +5266,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>100</v>
       </c>
@@ -5009,7 +5307,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>100</v>
       </c>
@@ -5050,7 +5348,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>100</v>
       </c>
@@ -5091,7 +5389,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>100</v>
       </c>
@@ -5132,7 +5430,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>100</v>
       </c>
@@ -5173,7 +5471,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>100</v>
       </c>
@@ -5214,7 +5512,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>100</v>
       </c>
@@ -5255,7 +5553,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>100</v>
       </c>
@@ -5296,7 +5594,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>100</v>
       </c>
@@ -5337,11 +5635,11 @@
         <v>238</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B74" s="19"/>
       <c r="C74" s="19"/>
     </row>
-    <row r="75" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A75" s="24" t="s">
         <v>131</v>
       </c>
@@ -5382,7 +5680,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>131</v>
       </c>
@@ -5423,7 +5721,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="77" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>131</v>
       </c>
@@ -5464,7 +5762,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="78" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>131</v>
       </c>
@@ -5505,7 +5803,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>131</v>
       </c>
@@ -5546,7 +5844,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>131</v>
       </c>
@@ -5587,12 +5885,12 @@
         <v>244</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B81" s="19"/>
       <c r="C81" s="19"/>
       <c r="H81" s="11"/>
     </row>
-    <row r="82" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>134</v>
       </c>
@@ -5633,7 +5931,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>134</v>
       </c>
@@ -5674,7 +5972,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>134</v>
       </c>
@@ -5715,7 +6013,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>134</v>
       </c>
@@ -5756,7 +6054,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="86" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A86" s="24" t="s">
         <v>396</v>
       </c>
@@ -5797,7 +6095,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="112" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>140</v>
       </c>
@@ -5838,11 +6136,11 @@
         <v>178</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B88" s="19"/>
       <c r="C88" s="19"/>
     </row>
-    <row r="89" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>131</v>
       </c>
@@ -5883,7 +6181,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="90" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>131</v>
       </c>
@@ -5924,7 +6222,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="91" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>131</v>
       </c>
@@ -5965,7 +6263,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>131</v>
       </c>
@@ -6006,7 +6304,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>131</v>
       </c>
@@ -6047,7 +6345,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="94" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>131</v>
       </c>
@@ -6088,10 +6386,10 @@
         <v>277</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="G95" s="8"/>
     </row>
-    <row r="96" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>286</v>
       </c>
@@ -6132,11 +6430,11 @@
         <v>395</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B97" s="19"/>
       <c r="C97" s="19"/>
     </row>
-    <row r="98" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>289</v>
       </c>
@@ -6177,7 +6475,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="100" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>301</v>
       </c>
@@ -6218,7 +6516,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="101" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>301</v>
       </c>
@@ -6259,7 +6557,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="102" spans="1:13" ht="176" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:13" ht="195" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>302</v>
       </c>
@@ -6300,11 +6598,11 @@
         <v>400</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B103" s="19"/>
       <c r="C103" s="19"/>
     </row>
-    <row r="104" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>315</v>
       </c>
@@ -6345,7 +6643,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="105" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>315</v>
       </c>
@@ -6386,7 +6684,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="106" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>315</v>
       </c>
@@ -6427,7 +6725,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="107" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>405</v>
       </c>
@@ -6468,7 +6766,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="108" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>330</v>
       </c>
@@ -6509,7 +6807,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="109" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>405</v>
       </c>
@@ -6550,7 +6848,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="110" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>405</v>
       </c>
@@ -6591,7 +6889,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="111" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>331</v>
       </c>
@@ -6632,7 +6930,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="112" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>405</v>
       </c>
@@ -6673,7 +6971,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="113" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>405</v>
       </c>
@@ -6714,11 +7012,11 @@
         <v>408</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B114" s="19"/>
       <c r="C114" s="19"/>
     </row>
-    <row r="115" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>343</v>
       </c>
@@ -6759,7 +7057,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="116" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>342</v>
       </c>
@@ -6800,7 +7098,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="117" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>342</v>
       </c>
@@ -6841,11 +7139,11 @@
         <v>346</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B118" s="19"/>
       <c r="C118" s="19"/>
     </row>
-    <row r="119" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A119" s="24" t="s">
         <v>349</v>
       </c>
@@ -6886,7 +7184,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="120" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>349</v>
       </c>
@@ -6927,7 +7225,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="121" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>349</v>
       </c>
@@ -6968,7 +7266,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="122" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>349</v>
       </c>
@@ -7009,7 +7307,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="123" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>349</v>
       </c>
@@ -7050,7 +7348,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="124" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>349</v>
       </c>
@@ -7091,7 +7389,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="125" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>349</v>
       </c>
@@ -7132,7 +7430,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="126" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>349</v>
       </c>
@@ -7173,7 +7471,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="127" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>349</v>
       </c>
@@ -7214,7 +7512,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="128" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>349</v>
       </c>
@@ -7255,7 +7553,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="129" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>349</v>
       </c>
@@ -7296,7 +7594,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="130" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>349</v>
       </c>
@@ -7337,7 +7635,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="131" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>349</v>
       </c>
@@ -7378,7 +7676,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="132" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>349</v>
       </c>
@@ -7419,7 +7717,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="133" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>349</v>
       </c>
@@ -7460,7 +7758,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="134" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>349</v>
       </c>
@@ -7501,7 +7799,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="135" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>349</v>
       </c>
@@ -7542,7 +7840,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="136" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>349</v>
       </c>
@@ -7583,7 +7881,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="137" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A137" s="26" t="s">
         <v>349</v>
       </c>
@@ -7624,7 +7922,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="138" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A138" s="23" t="s">
         <v>349</v>
       </c>
@@ -7665,7 +7963,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="139" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A139" s="23" t="s">
         <v>349</v>
       </c>
@@ -7706,7 +8004,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="140" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A140" s="23" t="s">
         <v>349</v>
       </c>
@@ -7747,7 +8045,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="141" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A141" s="23" t="s">
         <v>349</v>
       </c>
@@ -7788,7 +8086,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="142" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A142" s="23" t="s">
         <v>349</v>
       </c>
@@ -7829,7 +8127,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="143" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A143" s="23" t="s">
         <v>349</v>
       </c>
@@ -7870,7 +8168,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="144" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A144" s="23" t="s">
         <v>349</v>
       </c>
@@ -7911,7 +8209,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="145" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A145" s="23" t="s">
         <v>349</v>
       </c>
@@ -7952,7 +8250,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="146" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A146" s="23" t="s">
         <v>349</v>
       </c>
@@ -7993,7 +8291,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="147" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A147" s="23" t="s">
         <v>349</v>
       </c>
@@ -8034,7 +8332,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="148" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A148" s="23" t="s">
         <v>349</v>
       </c>
@@ -8075,7 +8373,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="149" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A149" s="23" t="s">
         <v>349</v>
       </c>
@@ -8116,7 +8414,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="150" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A150" s="23" t="s">
         <v>349</v>
       </c>
@@ -8157,7 +8455,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="151" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A151" s="23" t="s">
         <v>349</v>
       </c>
@@ -8198,7 +8496,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="152" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A152" s="23" t="s">
         <v>349</v>
       </c>
@@ -8239,7 +8537,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="153" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A153" s="23" t="s">
         <v>349</v>
       </c>
@@ -8280,7 +8578,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="154" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A154" s="23" t="s">
         <v>349</v>
       </c>
@@ -8321,12 +8619,12 @@
         <v>441</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="23"/>
       <c r="B155" s="19"/>
       <c r="C155" s="19"/>
     </row>
-    <row r="156" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>358</v>
       </c>
@@ -8367,7 +8665,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="157" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>358</v>
       </c>
@@ -8408,7 +8706,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="158" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>358</v>
       </c>
@@ -8449,7 +8747,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="159" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>358</v>
       </c>
@@ -8490,7 +8788,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="160" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>358</v>
       </c>
@@ -8531,7 +8829,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="161" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>358</v>
       </c>
@@ -8572,7 +8870,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="162" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>358</v>
       </c>
@@ -8613,7 +8911,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="163" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>358</v>
       </c>
@@ -8654,7 +8952,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="164" spans="1:13" ht="112" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>358</v>
       </c>
@@ -8695,12 +8993,12 @@
         <v>362</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B165" s="19"/>
       <c r="C165" s="19"/>
       <c r="D165" s="4"/>
     </row>
-    <row r="166" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>379</v>
       </c>
@@ -8741,12 +9039,12 @@
         <v>381</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B167" s="19"/>
       <c r="C167" s="19"/>
       <c r="D167" s="4"/>
     </row>
-    <row r="168" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A168" s="10" t="s">
         <v>451</v>
       </c>
@@ -8787,7 +9085,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="169" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A169" s="10" t="s">
         <v>451</v>
       </c>
@@ -8828,7 +9126,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="170" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A170" s="10" t="s">
         <v>451</v>
       </c>
@@ -8935,386 +9233,2274 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C17FE217-AB61-B742-BFE0-33900D1BEC91}">
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J71"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="17.1640625" customWidth="1"/>
-    <col min="3" max="3" width="53.33203125" customWidth="1"/>
-    <col min="4" max="4" width="29.1640625" customWidth="1"/>
-    <col min="5" max="5" width="30.5" customWidth="1"/>
-    <col min="6" max="7" width="17.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16.5" customWidth="1"/>
-    <col min="9" max="9" width="33.5" customWidth="1"/>
-    <col min="10" max="10" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="53.28515625" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" customWidth="1"/>
+    <col min="5" max="5" width="30.42578125" customWidth="1"/>
+    <col min="6" max="7" width="17.28515625" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" customWidth="1"/>
+    <col min="9" max="9" width="33.42578125" customWidth="1"/>
+    <col min="10" max="10" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="49" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="33" t="s">
         <v>494</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="E1" s="34" t="s">
         <v>495</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="F1" s="37" t="s">
         <v>496</v>
       </c>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="53"/>
-      <c r="J1" s="36"/>
-    </row>
-    <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="37" t="s">
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="27"/>
+    </row>
+    <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
         <v>491</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="28" t="s">
         <v>484</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="28" t="s">
         <v>483</v>
       </c>
-      <c r="D2" s="49"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="38" t="s">
+      <c r="D2" s="33"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="29" t="s">
         <v>460</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="G2" s="30" t="s">
         <v>497</v>
       </c>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="28" t="s">
         <v>461</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="I2" s="31" t="s">
         <v>489</v>
       </c>
-      <c r="J2" s="41" t="s">
+      <c r="J2" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E3" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F3" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E4" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F4" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E5" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F5" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E6" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F6" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F7" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F8" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F9" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="49" t="s">
         <v>486</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C10" s="16" t="s">
         <v>498</v>
       </c>
-      <c r="D3" s="44" t="s">
+      <c r="D10" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E10" s="47" t="s">
         <v>454</v>
       </c>
-      <c r="F3" s="46" t="s">
+      <c r="F10" s="48" t="s">
         <v>488</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="G10" s="49" t="s">
         <v>479</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="H10" s="49" t="s">
         <v>476</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="I10" s="50" t="s">
         <v>470</v>
       </c>
-      <c r="J3" s="29" t="s">
+      <c r="J10" s="51" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="27" t="s">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="49" t="s">
         <v>486</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C11" s="16" t="s">
         <v>498</v>
       </c>
-      <c r="D4" s="44" t="s">
+      <c r="D11" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="E4" s="45" t="s">
+      <c r="E11" s="47" t="s">
         <v>454</v>
       </c>
-      <c r="F4" s="46" t="s">
+      <c r="F11" s="48" t="s">
         <v>488</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G11" s="49" t="s">
         <v>479</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H11" s="49" t="s">
         <v>476</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I11" s="50" t="s">
         <v>471</v>
       </c>
-      <c r="J4" s="29" t="s">
+      <c r="J11" s="51" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="27" t="s">
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F12" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G12" t="s">
+        <v>481</v>
+      </c>
+      <c r="H12" t="s">
+        <v>478</v>
+      </c>
+      <c r="I12" t="s">
+        <v>474</v>
+      </c>
+      <c r="J12" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E13" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F13" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G13" t="s">
+        <v>481</v>
+      </c>
+      <c r="H13" t="s">
+        <v>478</v>
+      </c>
+      <c r="I13" t="s">
+        <v>473</v>
+      </c>
+      <c r="J13" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C14" s="54" t="s">
         <v>492</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="D14" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="E5" s="45" t="s">
+      <c r="E14" s="47" t="s">
         <v>454</v>
       </c>
-      <c r="F5" s="46" t="s">
+      <c r="F14" s="48" t="s">
         <v>488</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G14" s="49" t="s">
         <v>479</v>
       </c>
-      <c r="H5" s="27" t="s">
+      <c r="H14" s="49" t="s">
         <v>476</v>
       </c>
-      <c r="I5" s="28" t="s">
+      <c r="I14" s="50" t="s">
         <v>472</v>
       </c>
-      <c r="J5" s="29" t="s">
+      <c r="J14" s="51" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="27" t="s">
+    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C15" s="54" t="s">
         <v>492</v>
       </c>
-      <c r="D6" s="44" t="s">
+      <c r="D15" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="E6" s="45" t="s">
+      <c r="E15" s="47" t="s">
         <v>454</v>
       </c>
-      <c r="F6" s="46" t="s">
+      <c r="F15" s="48" t="s">
         <v>488</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G15" s="49" t="s">
         <v>479</v>
       </c>
-      <c r="H6" s="27" t="s">
+      <c r="H15" s="49" t="s">
         <v>476</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="I15" s="50" t="s">
         <v>473</v>
       </c>
-      <c r="J6" s="29" t="s">
+      <c r="J15" s="51" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="27" t="s">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E16" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F16" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G16" t="s">
+        <v>505</v>
+      </c>
+      <c r="H16" t="s">
+        <v>506</v>
+      </c>
+      <c r="I16" t="s">
+        <v>473</v>
+      </c>
+      <c r="J16" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E17" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F17" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G17" t="s">
+        <v>505</v>
+      </c>
+      <c r="H17" t="s">
+        <v>506</v>
+      </c>
+      <c r="I17" t="s">
+        <v>472</v>
+      </c>
+      <c r="J17" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E18" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F18" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G18" t="s">
+        <v>505</v>
+      </c>
+      <c r="H18" t="s">
+        <v>506</v>
+      </c>
+      <c r="I18" t="s">
+        <v>471</v>
+      </c>
+      <c r="J18" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>509</v>
+      </c>
+      <c r="C19" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E19" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F19" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G19" t="s">
+        <v>479</v>
+      </c>
+      <c r="H19" t="s">
+        <v>476</v>
+      </c>
+      <c r="I19" t="s">
+        <v>474</v>
+      </c>
+      <c r="J19" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>509</v>
+      </c>
+      <c r="C20" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E20" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F20" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G20" t="s">
+        <v>479</v>
+      </c>
+      <c r="H20" t="s">
+        <v>476</v>
+      </c>
+      <c r="I20" t="s">
+        <v>471</v>
+      </c>
+      <c r="J20" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>509</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E21" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F21" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G21" t="s">
+        <v>512</v>
+      </c>
+      <c r="H21" t="s">
+        <v>476</v>
+      </c>
+      <c r="I21" t="s">
+        <v>471</v>
+      </c>
+      <c r="J21" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>514</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E22" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F22" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G22" t="s">
+        <v>515</v>
+      </c>
+      <c r="H22" t="s">
+        <v>477</v>
+      </c>
+      <c r="I22" t="s">
+        <v>474</v>
+      </c>
+      <c r="J22" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" t="s">
+        <v>514</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E23" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F23" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G23" t="s">
+        <v>517</v>
+      </c>
+      <c r="H23" t="s">
+        <v>476</v>
+      </c>
+      <c r="I23" t="s">
+        <v>474</v>
+      </c>
+      <c r="J23" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" t="s">
+        <v>514</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E24" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F24" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G24" t="s">
+        <v>519</v>
+      </c>
+      <c r="H24" t="s">
+        <v>520</v>
+      </c>
+      <c r="I24" t="s">
+        <v>472</v>
+      </c>
+      <c r="J24" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" t="s">
+        <v>514</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F25" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G25" t="s">
+        <v>522</v>
+      </c>
+      <c r="H25" t="s">
+        <v>523</v>
+      </c>
+      <c r="I25" t="s">
+        <v>473</v>
+      </c>
+      <c r="J25" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" t="s">
+        <v>514</v>
+      </c>
+      <c r="C26" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E26" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F26" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G26" t="s">
+        <v>525</v>
+      </c>
+      <c r="H26" t="s">
+        <v>523</v>
+      </c>
+      <c r="I26" t="s">
+        <v>473</v>
+      </c>
+      <c r="J26" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" t="s">
+        <v>527</v>
+      </c>
+      <c r="C27" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E27" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F27" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G27" t="s">
+        <v>528</v>
+      </c>
+      <c r="H27" t="s">
+        <v>506</v>
+      </c>
+      <c r="I27" t="s">
+        <v>473</v>
+      </c>
+      <c r="J27" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" t="s">
+        <v>527</v>
+      </c>
+      <c r="C28" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E28" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F28" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G28" t="s">
+        <v>530</v>
+      </c>
+      <c r="H28" t="s">
+        <v>506</v>
+      </c>
+      <c r="I28" t="s">
+        <v>473</v>
+      </c>
+      <c r="J28" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" t="s">
+        <v>527</v>
+      </c>
+      <c r="C29" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E29" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F29" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G29" t="s">
+        <v>530</v>
+      </c>
+      <c r="H29" t="s">
+        <v>506</v>
+      </c>
+      <c r="I29" t="s">
+        <v>472</v>
+      </c>
+      <c r="J29" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" t="s">
+        <v>533</v>
+      </c>
+      <c r="C30" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E30" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F30" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G30" t="s">
+        <v>530</v>
+      </c>
+      <c r="H30" t="s">
+        <v>506</v>
+      </c>
+      <c r="I30" t="s">
+        <v>473</v>
+      </c>
+      <c r="J30" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" t="s">
+        <v>533</v>
+      </c>
+      <c r="C31" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E31" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F31" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G31" t="s">
+        <v>530</v>
+      </c>
+      <c r="H31" t="s">
+        <v>506</v>
+      </c>
+      <c r="I31" t="s">
+        <v>472</v>
+      </c>
+      <c r="J31" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" t="s">
+        <v>304</v>
+      </c>
+      <c r="C32" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E32" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F32" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G32" t="s">
+        <v>536</v>
+      </c>
+      <c r="H32" t="s">
+        <v>520</v>
+      </c>
+      <c r="I32" t="s">
+        <v>537</v>
+      </c>
+      <c r="J32" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" t="s">
+        <v>304</v>
+      </c>
+      <c r="C33" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E33" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F33" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G33" t="s">
+        <v>539</v>
+      </c>
+      <c r="H33" t="s">
+        <v>520</v>
+      </c>
+      <c r="I33" t="s">
+        <v>474</v>
+      </c>
+      <c r="J33" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34" t="s">
+        <v>304</v>
+      </c>
+      <c r="C34" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E34" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F34" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G34" t="s">
+        <v>481</v>
+      </c>
+      <c r="H34" t="s">
+        <v>478</v>
+      </c>
+      <c r="I34" t="s">
+        <v>474</v>
+      </c>
+      <c r="J34" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E35" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F35" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G35" t="s">
+        <v>479</v>
+      </c>
+      <c r="H35" t="s">
+        <v>476</v>
+      </c>
+      <c r="I35" t="s">
+        <v>542</v>
+      </c>
+      <c r="J35" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E36" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F36" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G36" t="s">
+        <v>479</v>
+      </c>
+      <c r="H36" t="s">
+        <v>476</v>
+      </c>
+      <c r="I36" t="s">
+        <v>471</v>
+      </c>
+      <c r="J36" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E37" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F37" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G37" t="s">
+        <v>545</v>
+      </c>
+      <c r="H37" t="s">
+        <v>476</v>
+      </c>
+      <c r="I37" t="s">
+        <v>542</v>
+      </c>
+      <c r="J37" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E38" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F38" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G38" t="s">
+        <v>545</v>
+      </c>
+      <c r="H38" t="s">
+        <v>476</v>
+      </c>
+      <c r="I38" t="s">
+        <v>471</v>
+      </c>
+      <c r="J38" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E39" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F39" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G39" t="s">
+        <v>480</v>
+      </c>
+      <c r="H39" t="s">
+        <v>477</v>
+      </c>
+      <c r="I39" t="s">
+        <v>474</v>
+      </c>
+      <c r="J39" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E40" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F40" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G40" t="s">
+        <v>547</v>
+      </c>
+      <c r="H40" t="s">
+        <v>523</v>
+      </c>
+      <c r="I40" t="s">
+        <v>470</v>
+      </c>
+      <c r="J40" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B41" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E41" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F41" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G41" t="s">
+        <v>479</v>
+      </c>
+      <c r="H41" t="s">
+        <v>476</v>
+      </c>
+      <c r="I41" t="s">
+        <v>473</v>
+      </c>
+      <c r="J41" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E42" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F42" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G42" t="s">
+        <v>545</v>
+      </c>
+      <c r="H42" t="s">
+        <v>476</v>
+      </c>
+      <c r="I42" t="s">
+        <v>473</v>
+      </c>
+      <c r="J42" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A43" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B43" t="s">
+        <v>550</v>
+      </c>
+      <c r="C43" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E43" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F43" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G43" t="s">
+        <v>539</v>
+      </c>
+      <c r="H43" t="s">
+        <v>520</v>
+      </c>
+      <c r="I43" t="s">
+        <v>473</v>
+      </c>
+      <c r="J43" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" t="s">
+        <v>550</v>
+      </c>
+      <c r="C44" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E44" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F44" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G44" t="s">
+        <v>539</v>
+      </c>
+      <c r="H44" t="s">
+        <v>520</v>
+      </c>
+      <c r="I44" t="s">
+        <v>473</v>
+      </c>
+      <c r="J44" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B45" t="s">
+        <v>550</v>
+      </c>
+      <c r="C45" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E45" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F45" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G45" t="s">
+        <v>539</v>
+      </c>
+      <c r="H45" t="s">
+        <v>520</v>
+      </c>
+      <c r="I45" t="s">
+        <v>471</v>
+      </c>
+      <c r="J45" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" t="s">
+        <v>550</v>
+      </c>
+      <c r="C46" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E46" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F46" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G46" t="s">
+        <v>515</v>
+      </c>
+      <c r="H46" t="s">
+        <v>477</v>
+      </c>
+      <c r="I46" t="s">
+        <v>471</v>
+      </c>
+      <c r="J46" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B47" t="s">
+        <v>550</v>
+      </c>
+      <c r="C47" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E47" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F47" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G47" t="s">
+        <v>530</v>
+      </c>
+      <c r="H47" t="s">
+        <v>506</v>
+      </c>
+      <c r="I47" t="s">
+        <v>542</v>
+      </c>
+      <c r="J47" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B48" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E48" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F48" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G48" t="s">
+        <v>556</v>
+      </c>
+      <c r="H48" t="s">
+        <v>520</v>
+      </c>
+      <c r="I48" t="s">
+        <v>473</v>
+      </c>
+      <c r="J48" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B49" t="s">
+        <v>132</v>
+      </c>
+      <c r="C49" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E49" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F49" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G49" t="s">
+        <v>556</v>
+      </c>
+      <c r="H49" t="s">
+        <v>520</v>
+      </c>
+      <c r="I49" t="s">
+        <v>474</v>
+      </c>
+      <c r="J49" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B50" t="s">
+        <v>360</v>
+      </c>
+      <c r="C50" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E50" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F50" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G50" t="s">
+        <v>481</v>
+      </c>
+      <c r="H50" t="s">
+        <v>478</v>
+      </c>
+      <c r="I50" t="s">
+        <v>473</v>
+      </c>
+      <c r="J50" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B51" t="s">
+        <v>360</v>
+      </c>
+      <c r="C51" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E51" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F51" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G51" t="s">
+        <v>515</v>
+      </c>
+      <c r="H51" t="s">
+        <v>477</v>
+      </c>
+      <c r="I51" t="s">
+        <v>474</v>
+      </c>
+      <c r="J51" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B52" t="s">
+        <v>561</v>
+      </c>
+      <c r="C52" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E52" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F52" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G52" t="s">
+        <v>515</v>
+      </c>
+      <c r="H52" t="s">
+        <v>477</v>
+      </c>
+      <c r="I52" t="s">
+        <v>474</v>
+      </c>
+      <c r="J52" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B53" t="s">
+        <v>561</v>
+      </c>
+      <c r="C53" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E53" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F53" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G53" t="s">
+        <v>505</v>
+      </c>
+      <c r="H53" t="s">
+        <v>506</v>
+      </c>
+      <c r="I53" t="s">
+        <v>474</v>
+      </c>
+      <c r="J53" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B54" t="s">
+        <v>561</v>
+      </c>
+      <c r="C54" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D54" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E54" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F54" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G54" t="s">
+        <v>479</v>
+      </c>
+      <c r="H54" t="s">
+        <v>476</v>
+      </c>
+      <c r="I54" t="s">
+        <v>470</v>
+      </c>
+      <c r="J54" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55" t="s">
+        <v>561</v>
+      </c>
+      <c r="C55" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D55" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E55" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F55" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G55" t="s">
+        <v>512</v>
+      </c>
+      <c r="H55" t="s">
+        <v>476</v>
+      </c>
+      <c r="I55" t="s">
+        <v>470</v>
+      </c>
+      <c r="J55" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A56" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" t="s">
+        <v>561</v>
+      </c>
+      <c r="C56" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E56" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F56" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G56" t="s">
+        <v>530</v>
+      </c>
+      <c r="H56" t="s">
+        <v>506</v>
+      </c>
+      <c r="I56" t="s">
+        <v>470</v>
+      </c>
+      <c r="J56" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" t="s">
+        <v>567</v>
+      </c>
+      <c r="C57" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E57" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F57" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G57" t="s">
+        <v>479</v>
+      </c>
+      <c r="H57" t="s">
+        <v>476</v>
+      </c>
+      <c r="I57" t="s">
+        <v>473</v>
+      </c>
+      <c r="J57" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" t="s">
+        <v>569</v>
+      </c>
+      <c r="C58" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D58" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E58" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F58" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G58" t="s">
+        <v>556</v>
+      </c>
+      <c r="H58" t="s">
+        <v>520</v>
+      </c>
+      <c r="I58" t="s">
+        <v>473</v>
+      </c>
+      <c r="J58" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A59" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" t="s">
+        <v>571</v>
+      </c>
+      <c r="C59" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E59" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F59" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G59" t="s">
+        <v>572</v>
+      </c>
+      <c r="H59" t="s">
+        <v>573</v>
+      </c>
+      <c r="I59" t="s">
+        <v>542</v>
+      </c>
+      <c r="J59" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" t="s">
+        <v>320</v>
+      </c>
+      <c r="C60" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D60" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E60" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F60" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G60" t="s">
+        <v>515</v>
+      </c>
+      <c r="H60" t="s">
+        <v>477</v>
+      </c>
+      <c r="I60" t="s">
+        <v>474</v>
+      </c>
+      <c r="J60" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B61" t="s">
+        <v>320</v>
+      </c>
+      <c r="C61" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E61" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F61" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G61" t="s">
+        <v>480</v>
+      </c>
+      <c r="H61" t="s">
+        <v>477</v>
+      </c>
+      <c r="I61" t="s">
+        <v>474</v>
+      </c>
+      <c r="J61" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B62" t="s">
+        <v>320</v>
+      </c>
+      <c r="C62" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D62" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E62" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F62" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G62" t="s">
+        <v>481</v>
+      </c>
+      <c r="H62" t="s">
+        <v>478</v>
+      </c>
+      <c r="I62" t="s">
+        <v>474</v>
+      </c>
+      <c r="J62" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" t="s">
+        <v>320</v>
+      </c>
+      <c r="C63" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E63" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F63" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G63" t="s">
+        <v>578</v>
+      </c>
+      <c r="H63" t="s">
+        <v>579</v>
+      </c>
+      <c r="I63" t="s">
+        <v>472</v>
+      </c>
+      <c r="J63" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A64" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" t="s">
+        <v>291</v>
+      </c>
+      <c r="C64" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E64" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F64" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G64" t="s">
+        <v>481</v>
+      </c>
+      <c r="H64" t="s">
+        <v>478</v>
+      </c>
+      <c r="I64" t="s">
+        <v>474</v>
+      </c>
+      <c r="J64" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A65" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B65" t="s">
+        <v>581</v>
+      </c>
+      <c r="C65" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D65" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E65" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F65" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G65" t="s">
+        <v>582</v>
+      </c>
+      <c r="H65" t="s">
+        <v>476</v>
+      </c>
+      <c r="I65" t="s">
+        <v>473</v>
+      </c>
+      <c r="J65" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B66" t="s">
+        <v>584</v>
+      </c>
+      <c r="C66" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E66" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F66" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G66" t="s">
+        <v>480</v>
+      </c>
+      <c r="H66" t="s">
+        <v>477</v>
+      </c>
+      <c r="I66" t="s">
+        <v>474</v>
+      </c>
+      <c r="J66" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B67" t="s">
+        <v>584</v>
+      </c>
+      <c r="C67" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E67" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F67" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G67" t="s">
+        <v>481</v>
+      </c>
+      <c r="H67" t="s">
+        <v>478</v>
+      </c>
+      <c r="I67" t="s">
+        <v>474</v>
+      </c>
+      <c r="J67" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A68" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" t="s">
+        <v>39</v>
+      </c>
+      <c r="C68" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E68" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F68" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G68" t="s">
+        <v>480</v>
+      </c>
+      <c r="H68" t="s">
+        <v>477</v>
+      </c>
+      <c r="I68" t="s">
+        <v>470</v>
+      </c>
+      <c r="J68" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A69" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D69" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="E69" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="F69" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="G69" t="s">
+        <v>588</v>
+      </c>
+      <c r="H69" t="s">
+        <v>589</v>
+      </c>
+      <c r="I69" t="s">
+        <v>470</v>
+      </c>
+      <c r="J69" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A70" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B70" s="49" t="s">
         <v>378</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C70" s="54" t="s">
         <v>493</v>
       </c>
-      <c r="D7" s="44" t="s">
+      <c r="D70" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="E7" s="45" t="s">
+      <c r="E70" s="47" t="s">
         <v>454</v>
       </c>
-      <c r="F7" s="46" t="s">
+      <c r="F70" s="48" t="s">
         <v>488</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G70" s="49" t="s">
         <v>480</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="H70" s="49" t="s">
         <v>477</v>
       </c>
-      <c r="I7" s="28" t="s">
+      <c r="I70" s="50" t="s">
         <v>474</v>
       </c>
-      <c r="J7" s="29" t="s">
+      <c r="J70" s="51" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="27" t="s">
+    <row r="71" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A71" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="B71" s="49" t="s">
         <v>340</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C71" s="56" t="s">
         <v>485</v>
       </c>
-      <c r="D8" s="44" t="s">
+      <c r="D71" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="E8" s="45" t="s">
+      <c r="E71" s="47" t="s">
         <v>454</v>
       </c>
-      <c r="F8" s="46" t="s">
+      <c r="F71" s="48" t="s">
         <v>488</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G71" s="49" t="s">
         <v>481</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H71" s="49" t="s">
         <v>478</v>
       </c>
-      <c r="I8" s="28" t="s">
+      <c r="I71" s="50" t="s">
         <v>474</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="J71" s="51" t="s">
         <v>467</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="27" t="s">
-        <v>487</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>485</v>
-      </c>
-      <c r="D9" s="44" t="s">
-        <v>453</v>
-      </c>
-      <c r="E9" s="45" t="s">
-        <v>454</v>
-      </c>
-      <c r="F9" s="46" t="s">
-        <v>488</v>
-      </c>
-      <c r="G9" s="27" t="s">
-        <v>482</v>
-      </c>
-      <c r="H9" s="27" t="s">
-        <v>476</v>
-      </c>
-      <c r="I9" s="28" t="s">
-        <v>471</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="27" t="s">
-        <v>487</v>
-      </c>
-      <c r="C10" s="27" t="s">
-        <v>485</v>
-      </c>
-      <c r="D10" s="44" t="s">
-        <v>453</v>
-      </c>
-      <c r="E10" s="45" t="s">
-        <v>454</v>
-      </c>
-      <c r="F10" s="46" t="s">
-        <v>488</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>482</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>476</v>
-      </c>
-      <c r="I10" s="28" t="s">
-        <v>475</v>
-      </c>
-      <c r="J10" s="29" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>487</v>
-      </c>
-      <c r="C11" s="27" t="s">
-        <v>485</v>
-      </c>
-      <c r="D11" s="44" t="s">
-        <v>453</v>
-      </c>
-      <c r="E11" s="45" t="s">
-        <v>454</v>
-      </c>
-      <c r="F11" s="46" t="s">
-        <v>488</v>
-      </c>
-      <c r="G11" s="27" t="s">
-        <v>481</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>478</v>
-      </c>
-      <c r="I11" s="28" t="s">
-        <v>471</v>
-      </c>
-      <c r="J11" s="29" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="27" t="s">
-        <v>487</v>
-      </c>
-      <c r="C12" s="27" t="s">
-        <v>485</v>
-      </c>
-      <c r="D12" s="44" t="s">
-        <v>453</v>
-      </c>
-      <c r="E12" s="45" t="s">
-        <v>454</v>
-      </c>
-      <c r="F12" s="46" t="s">
-        <v>488</v>
-      </c>
-      <c r="G12" s="27" t="s">
-        <v>481</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>478</v>
-      </c>
-      <c r="I12" s="28" t="s">
-        <v>475</v>
-      </c>
-      <c r="J12" s="29" t="s">
-        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -9325,10 +11511,11 @@
     <mergeCell ref="F1:I1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{E7EBFD69-AB42-1D4C-B09F-BC06AC0B1941}"/>
-    <hyperlink ref="C4" r:id="rId2" xr:uid="{19F34C30-987C-8A4F-A400-AB95B6919C72}"/>
-    <hyperlink ref="C5" r:id="rId3" xr:uid="{EB4AB897-0111-9A4F-A836-A7EA2313DA8B}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{849BF08E-F4EA-6945-93EA-AD080F320746}"/>
+    <hyperlink ref="C15" r:id="rId1" xr:uid="{294DB162-98E0-4B40-B781-02251F467A27}"/>
+    <hyperlink ref="C11" r:id="rId2" xr:uid="{8C07C59C-DA86-4C8D-9DA6-4A5AD6B80303}"/>
+    <hyperlink ref="C10" r:id="rId3" xr:uid="{B5671DF9-3065-42E2-9796-B313A496FC76}"/>
+    <hyperlink ref="C14" r:id="rId4" xr:uid="{E53E5D07-BD2D-4B6C-B0A0-EF6A87F85B42}"/>
+    <hyperlink ref="C70" r:id="rId5" xr:uid="{AC230D2C-F23B-4440-90A7-C101B0AB6EAB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9337,18 +11524,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0B35E6D-763F-4C40-91D2-473BE7766F62}">
   <dimension ref="A1:B22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5" customWidth="1"/>
-    <col min="2" max="2" width="105.1640625" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="2" width="105.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>145</v>
       </c>
@@ -9356,7 +11543,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -9364,7 +11551,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -9372,7 +11559,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>149</v>
       </c>
@@ -9380,7 +11567,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>151</v>
       </c>
@@ -9388,7 +11575,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>80</v>
       </c>
@@ -9396,7 +11583,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -9404,7 +11591,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>155</v>
       </c>
@@ -9412,7 +11599,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>157</v>
       </c>
@@ -9420,7 +11607,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -9428,7 +11615,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -9436,7 +11623,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -9444,7 +11631,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>76</v>
       </c>
@@ -9452,7 +11639,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>40</v>
       </c>
@@ -9460,7 +11647,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>164</v>
       </c>
@@ -9468,7 +11655,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>166</v>
       </c>
@@ -9476,7 +11663,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>168</v>
       </c>
@@ -9484,7 +11671,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>170</v>
       </c>
@@ -9492,7 +11679,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>454</v>
       </c>
@@ -9500,7 +11687,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>453</v>
       </c>
@@ -9752,6 +11939,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="80b53ead-ac38-442a-b597-5a0e2e0802cd">
@@ -9760,15 +11956,6 @@
     <TaxCatchAll xmlns="5ec1cc48-4270-4222-9ed5-54ce9e59d47b" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9791,6 +11978,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B1B5D08-A2EB-4F47-BA81-DA28AA2A09F4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66AF2240-620B-4312-9739-CAF731E4A98F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9799,12 +11994,4 @@
     <ds:schemaRef ds:uri="5ec1cc48-4270-4222-9ed5-54ce9e59d47b"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B1B5D08-A2EB-4F47-BA81-DA28AA2A09F4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>